<commit_message>
Harden backtest provenance and safety foundations
</commit_message>
<xml_diff>
--- a/reports/debug/trade_filter_statistics.xlsx
+++ b/reports/debug/trade_filter_statistics.xlsx
@@ -442,81 +442,81 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>413</v>
+        <v>93</v>
       </c>
       <c r="C2" t="n">
-        <v>82.59999999999999</v>
+        <v>66.42857142857143</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Rejected by insufficient data</t>
+          <t>Rejected by evaluation schedule</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C3" t="n">
-        <v>17.4</v>
+        <v>59.28571428571428</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Rejected by evaluation schedule</t>
+          <t>Rejected by insufficient data</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>20</v>
+        <v>47</v>
       </c>
       <c r="C4" t="n">
-        <v>4</v>
+        <v>33.57142857142857</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rejected by regime</t>
+          <t>Rejected by news</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Rejected by risk management</t>
+          <t>Rejected by regime</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>2.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Rejected by probability threshold</t>
+          <t>Rejected by ML confidence</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Rejected by news</t>
+          <t>Rejected by probability threshold</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -542,7 +542,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Rejected by ML confidence</t>
+          <t>Rejected by position sizing</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -555,7 +555,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Rejected by position sizing</t>
+          <t>Rejected by risk management</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -576,7 +576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
@@ -608,7 +608,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>20</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4">
@@ -628,27 +628,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>REJECTED_NO_CANDIDATE</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>REJECTED_RISK_MANAGEMENT</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>2</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -662,7 +642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -685,11 +665,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Bearish high volatility</t>
+          <t>NOT_EVALUATED</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -698,92 +678,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Bearish low volatility</t>
+          <t>Sideways low volatility</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>40</v>
+        <v>93</v>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Bullish high volatility</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>52</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Bullish low volatility</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>40</v>
-      </c>
-      <c r="C5" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Liquidity-trap/fake-breakout</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>13</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>NOT_EVALUATED</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>87</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Sideways high volatility</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>119</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Sideways low volatility</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>94</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>